<commit_message>
quản lý dữ liệu điểm xét tuyển
</commit_message>
<xml_diff>
--- a/data/import_phuong_thuc.xlsx
+++ b/data/import_phuong_thuc.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\chat-bot-tuyen-sinh\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5DF41C1-3C4C-498E-B646-101F0DC067ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1AB9C53-BE6B-4E0A-969F-4E4470F17741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,46 +20,43 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Mã Phương Thức</t>
   </si>
   <si>
-    <t>100</t>
-  </si>
-  <si>
-    <t>Phương thức 2: Xét tuyển bằng kết quả thi tốt nghiệp THPT năm 2026</t>
-  </si>
-  <si>
-    <t>200</t>
-  </si>
-  <si>
-    <t>Phương thức 3: Xét tuyển bằng học bạ THPT</t>
-  </si>
-  <si>
     <t>301</t>
   </si>
   <si>
-    <t>Phương thức 1: Xét tuyển thẳng và ưu tiên xét tuyển</t>
-  </si>
-  <si>
-    <t>405</t>
-  </si>
-  <si>
-    <t>Phương thức 4: Xét tuyển kết hợp thi năng khiếu</t>
-  </si>
-  <si>
     <t>Năm</t>
   </si>
   <si>
     <t>Tên Phương Thức</t>
+  </si>
+  <si>
+    <t>Điểm trúng tuyển sử dụng kết quả thi tốt nghiệp THPT</t>
+  </si>
+  <si>
+    <t>Điểm trúng tuyển sử dụng kết quả học tập cấp THPT (học bạ)</t>
+  </si>
+  <si>
+    <t>Điểm trúng tuyển theo kết quả Kỳ thi đánh giá tư duy và năng lực</t>
+  </si>
+  <si>
+    <t>Điểm trúng tuyển kết hợp kết quả thi tốt nghiệp THPT với điểm thi năng khiếu</t>
+  </si>
+  <si>
+    <t>Điểm trúng tuyển kết hợp kết quả học tập cấp THPT với điểm thi năng khiếu</t>
+  </si>
+  <si>
+    <t>Xét tuyển thẳng và ưu tiên xét tuyển</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -84,16 +81,30 @@
       <charset val="163"/>
       <scheme val="major"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="163"/>
+      <scheme val="major"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -116,16 +127,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -430,54 +474,54 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.19921875" customWidth="1"/>
-    <col min="3" max="3" width="48.8984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>2026</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>2</v>
+      <c r="B2" s="3">
+        <v>100</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2026</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>4</v>
+      <c r="B3" s="5">
+        <v>200</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>2026</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="B4" s="3">
+        <v>402</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>6</v>
       </c>
     </row>
@@ -485,11 +529,33 @@
       <c r="A5" s="2">
         <v>2026</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="5">
+        <v>405</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="2" t="s">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>2026</v>
+      </c>
+      <c r="B6" s="7">
+        <v>406</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>2026</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>